<commit_message>
Add backend API contract and shared app interfaces
- docs/API.md: Apps Script backend contract (Google ID token login,
  signed sessions, permissions, sheet mapping, money/time rules,
  idempotency, optimistic concurrency, error codes).
- Flutter: app config, ApiException, BackendApi interface, data models,
  number parsing/formatting, AuthController interface, AppScope.
- Sheet: add the «محذوف» status for removed packaging draft items.
- Add google_sign_in, http, flutter_secure_storage and uuid packages.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FLj5X5gRSQBQNx2yMBbcW4
</commit_message>
<xml_diff>
--- a/sheets/rumman-calculator-template.xlsx
+++ b/sheets/rumman-calculator-template.xlsx
@@ -41406,9 +41406,12 @@
     <cfRule type="cellIs" priority="2" operator="equal" dxfId="6">
       <formula>"غير مكتمل"</formula>
     </cfRule>
+    <cfRule type="cellIs" priority="3" operator="equal" dxfId="8">
+      <formula>"محذوف"</formula>
+    </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A4:L303">
-    <cfRule type="expression" priority="3" dxfId="2">
+    <cfRule type="expression" priority="4" dxfId="2">
       <formula>AND(MOD(ROW(),2)=1,$A4&lt;&gt;"")</formula>
     </cfRule>
   </conditionalFormatting>
@@ -41417,7 +41420,7 @@
       <formula1>"قطعة,رزمة,لفة,رول,كرتونة,كغ"</formula1>
     </dataValidation>
     <dataValidation sqref="I4:I303" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="قيمة غير صحيحة" error="اختر قيمة من القائمة." type="list">
-      <formula1>"مكتمل,غير مكتمل"</formula1>
+      <formula1>"مكتمل,غير مكتمل,محذوف"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>